<commit_message>
fix(demo): corrige les valeurs Nature/Type de gain invalides dans les impacts
L'import Excel n'accepte que "CAPEX", "OPEX récurrent", "One-off" pour la
colonne Nature (4 lignes utilisaient "Chiffre d'affaires récurrent") et
"Réduction de coût", "Augmentation du CA", "Impact BFR" pour Type de gain
(4 lignes utilisaient "Amélioration du prix") — voir lib/leverExcelImport.ts.
Corrige les 8 impacts liés aux leviers de pricing/revenue management.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo/leviers_demo.xlsx
+++ b/demo/leviers_demo.xlsx
@@ -9685,7 +9685,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Chiffre d'affaires récurrent</t>
+          <t>OPEX récurrent</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -9696,7 +9696,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Amélioration du prix</t>
+          <t>Augmentation du CA</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -10330,7 +10330,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Chiffre d'affaires récurrent</t>
+          <t>OPEX récurrent</t>
         </is>
       </c>
       <c r="E25" t="n">
@@ -10341,7 +10341,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Amélioration du prix</t>
+          <t>Augmentation du CA</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -11068,7 +11068,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Chiffre d'affaires récurrent</t>
+          <t>OPEX récurrent</t>
         </is>
       </c>
       <c r="E41" t="n">
@@ -11079,7 +11079,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Amélioration du prix</t>
+          <t>Augmentation du CA</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -11806,7 +11806,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Chiffre d'affaires récurrent</t>
+          <t>OPEX récurrent</t>
         </is>
       </c>
       <c r="E57" t="n">
@@ -11817,7 +11817,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Amélioration du prix</t>
+          <t>Augmentation du CA</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">

</xml_diff>

<commit_message>
fix(demo): corrige les valeurs Nature/Type de gain invalides dans les impacts (#56)
L'import Excel n'accepte que "CAPEX", "OPEX récurrent", "One-off" pour la
colonne Nature (4 lignes utilisaient "Chiffre d'affaires récurrent") et
"Réduction de coût", "Augmentation du CA", "Impact BFR" pour Type de gain
(4 lignes utilisaient "Amélioration du prix") — voir lib/leverExcelImport.ts.
Corrige les 8 impacts liés aux leviers de pricing/revenue management.

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo/leviers_demo.xlsx
+++ b/demo/leviers_demo.xlsx
@@ -9685,7 +9685,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Chiffre d'affaires récurrent</t>
+          <t>OPEX récurrent</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -9696,7 +9696,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Amélioration du prix</t>
+          <t>Augmentation du CA</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -10330,7 +10330,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Chiffre d'affaires récurrent</t>
+          <t>OPEX récurrent</t>
         </is>
       </c>
       <c r="E25" t="n">
@@ -10341,7 +10341,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Amélioration du prix</t>
+          <t>Augmentation du CA</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -11068,7 +11068,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Chiffre d'affaires récurrent</t>
+          <t>OPEX récurrent</t>
         </is>
       </c>
       <c r="E41" t="n">
@@ -11079,7 +11079,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Amélioration du prix</t>
+          <t>Augmentation du CA</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -11806,7 +11806,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Chiffre d'affaires récurrent</t>
+          <t>OPEX récurrent</t>
         </is>
       </c>
       <c r="E57" t="n">
@@ -11817,7 +11817,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Amélioration du prix</t>
+          <t>Augmentation du CA</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">

</xml_diff>

<commit_message>
fix(demo): align generated lever/action dates with their status
Lever end dates could fall after "today" for a lever already marked
"Réalisé" (or before "today" for one still "Identifié"), which made
the date-driven "Réalisé à date" calculation correctly show €0K
despite a 100% status — a demo-data staleness issue flagged during
the ACME/ICES consistency audit, not a calculation bug. Dates are now
chosen per status (Réalisé ends before DEMO_TODAY, Identifié/Planifié
start after it, Exécuté straddles it), still fully deterministic.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo/leviers_demo.xlsx
+++ b/demo/leviers_demo.xlsx
@@ -534,10 +534,10 @@
         <v>COGS</v>
       </c>
       <c r="P2" t="str">
-        <v>2026-01-01</v>
+        <v>2026-11-01</v>
       </c>
       <c r="Q2" t="str">
-        <v>2026-06-28</v>
+        <v>2027-04-28</v>
       </c>
       <c r="R2" t="str">
         <v>Identifié</v>
@@ -620,10 +620,10 @@
         <v>COGS</v>
       </c>
       <c r="P3" t="str">
-        <v>2026-02-01</v>
+        <v>2026-12-01</v>
       </c>
       <c r="Q3" t="str">
-        <v>2026-08-28</v>
+        <v>2027-06-28</v>
       </c>
       <c r="R3" t="str">
         <v>Validé</v>
@@ -706,10 +706,10 @@
         <v>GA</v>
       </c>
       <c r="P4" t="str">
-        <v>2026-03-01</v>
+        <v>2026-11-01</v>
       </c>
       <c r="Q4" t="str">
-        <v>2026-10-28</v>
+        <v>2027-06-28</v>
       </c>
       <c r="R4" t="str">
         <v>Planifié</v>
@@ -795,7 +795,7 @@
         <v>2026-04-01</v>
       </c>
       <c r="Q5" t="str">
-        <v>2026-12-28</v>
+        <v>2027-02-28</v>
       </c>
       <c r="R5" t="str">
         <v>Exécuté</v>
@@ -881,7 +881,7 @@
         <v>2026-05-01</v>
       </c>
       <c r="Q6" t="str">
-        <v>2027-02-28</v>
+        <v>2026-07-28</v>
       </c>
       <c r="R6" t="str">
         <v>Réalisé</v>
@@ -964,10 +964,10 @@
         <v>COGS</v>
       </c>
       <c r="P7" t="str">
-        <v>2026-06-01</v>
+        <v>2027-01-01</v>
       </c>
       <c r="Q7" t="str">
-        <v>2027-04-28</v>
+        <v>2028-11-28</v>
       </c>
       <c r="R7" t="str">
         <v>Identifié</v>
@@ -1050,10 +1050,10 @@
         <v>GA</v>
       </c>
       <c r="P8" t="str">
-        <v>2026-07-01</v>
+        <v>2026-11-01</v>
       </c>
       <c r="Q8" t="str">
-        <v>2027-06-28</v>
+        <v>2027-04-28</v>
       </c>
       <c r="R8" t="str">
         <v>Validé</v>
@@ -1136,10 +1136,10 @@
         <v>GA</v>
       </c>
       <c r="P9" t="str">
-        <v>2026-08-01</v>
+        <v>2026-10-01</v>
       </c>
       <c r="Q9" t="str">
-        <v>2027-08-28</v>
+        <v>2027-04-28</v>
       </c>
       <c r="R9" t="str">
         <v>Planifié</v>
@@ -1222,10 +1222,10 @@
         <v>COGS</v>
       </c>
       <c r="P10" t="str">
-        <v>2026-09-01</v>
+        <v>2026-01-01</v>
       </c>
       <c r="Q10" t="str">
-        <v>2027-02-28</v>
+        <v>2026-10-28</v>
       </c>
       <c r="R10" t="str">
         <v>Exécuté</v>
@@ -1308,10 +1308,10 @@
         <v>COGS</v>
       </c>
       <c r="P11" t="str">
-        <v>2026-10-01</v>
+        <v>2026-03-01</v>
       </c>
       <c r="Q11" t="str">
-        <v>2027-04-28</v>
+        <v>2026-06-28</v>
       </c>
       <c r="R11" t="str">
         <v>Réalisé</v>
@@ -1394,10 +1394,10 @@
         <v>GA</v>
       </c>
       <c r="P12" t="str">
-        <v>2026-01-01</v>
+        <v>2026-12-01</v>
       </c>
       <c r="Q12" t="str">
-        <v>2026-08-28</v>
+        <v>2027-09-28</v>
       </c>
       <c r="R12" t="str">
         <v>Identifié</v>
@@ -1480,10 +1480,10 @@
         <v>REV</v>
       </c>
       <c r="P13" t="str">
-        <v>2026-02-01</v>
+        <v>2027-01-01</v>
       </c>
       <c r="Q13" t="str">
-        <v>2026-10-28</v>
+        <v>2028-11-28</v>
       </c>
       <c r="R13" t="str">
         <v>Validé</v>
@@ -1566,10 +1566,10 @@
         <v>SGA</v>
       </c>
       <c r="P14" t="str">
-        <v>2026-03-01</v>
+        <v>2026-09-01</v>
       </c>
       <c r="Q14" t="str">
-        <v>2026-12-28</v>
+        <v>2027-02-28</v>
       </c>
       <c r="R14" t="str">
         <v>Planifié</v>
@@ -1652,7 +1652,7 @@
         <v>COGS</v>
       </c>
       <c r="P15" t="str">
-        <v>2026-04-01</v>
+        <v>2026-06-01</v>
       </c>
       <c r="Q15" t="str">
         <v>2027-02-28</v>
@@ -1738,10 +1738,10 @@
         <v>GA</v>
       </c>
       <c r="P16" t="str">
-        <v>2026-05-01</v>
+        <v>2026-01-01</v>
       </c>
       <c r="Q16" t="str">
-        <v>2027-04-28</v>
+        <v>2026-05-28</v>
       </c>
       <c r="R16" t="str">
         <v>Réalisé</v>
@@ -1824,10 +1824,10 @@
         <v>GA</v>
       </c>
       <c r="P17" t="str">
-        <v>2026-06-01</v>
+        <v>2026-11-01</v>
       </c>
       <c r="Q17" t="str">
-        <v>2027-06-28</v>
+        <v>2027-07-28</v>
       </c>
       <c r="R17" t="str">
         <v>Identifié</v>
@@ -1910,10 +1910,10 @@
         <v>COGS</v>
       </c>
       <c r="P18" t="str">
-        <v>2026-07-01</v>
+        <v>2026-12-01</v>
       </c>
       <c r="Q18" t="str">
-        <v>2026-12-28</v>
+        <v>2027-09-28</v>
       </c>
       <c r="R18" t="str">
         <v>Validé</v>
@@ -1996,10 +1996,10 @@
         <v>COGS</v>
       </c>
       <c r="P19" t="str">
-        <v>2026-08-01</v>
+        <v>2026-11-01</v>
       </c>
       <c r="Q19" t="str">
-        <v>2027-02-28</v>
+        <v>2027-09-28</v>
       </c>
       <c r="R19" t="str">
         <v>Planifié</v>
@@ -2082,10 +2082,10 @@
         <v>GA</v>
       </c>
       <c r="P20" t="str">
-        <v>2026-09-01</v>
+        <v>2026-03-01</v>
       </c>
       <c r="Q20" t="str">
-        <v>2027-04-28</v>
+        <v>2026-10-28</v>
       </c>
       <c r="R20" t="str">
         <v>Exécuté</v>
@@ -2168,10 +2168,10 @@
         <v>REV</v>
       </c>
       <c r="P21" t="str">
-        <v>2026-10-01</v>
+        <v>2026-01-01</v>
       </c>
       <c r="Q21" t="str">
-        <v>2027-06-28</v>
+        <v>2026-06-28</v>
       </c>
       <c r="R21" t="str">
         <v>Réalisé</v>
@@ -2254,10 +2254,10 @@
         <v>SGA</v>
       </c>
       <c r="P22" t="str">
-        <v>2026-01-01</v>
+        <v>2027-01-01</v>
       </c>
       <c r="Q22" t="str">
-        <v>2026-10-28</v>
+        <v>2028-08-28</v>
       </c>
       <c r="R22" t="str">
         <v>Identifié</v>
@@ -2340,10 +2340,10 @@
         <v>COGS</v>
       </c>
       <c r="P23" t="str">
-        <v>2026-02-01</v>
+        <v>2026-11-01</v>
       </c>
       <c r="Q23" t="str">
-        <v>2026-12-28</v>
+        <v>2027-07-28</v>
       </c>
       <c r="R23" t="str">
         <v>Validé</v>
@@ -2426,10 +2426,10 @@
         <v>GA</v>
       </c>
       <c r="P24" t="str">
-        <v>2026-03-01</v>
+        <v>2026-10-01</v>
       </c>
       <c r="Q24" t="str">
-        <v>2027-02-28</v>
+        <v>2027-07-28</v>
       </c>
       <c r="R24" t="str">
         <v>Planifié</v>
@@ -2512,10 +2512,10 @@
         <v>GA</v>
       </c>
       <c r="P25" t="str">
-        <v>2026-04-01</v>
+        <v>2026-08-01</v>
       </c>
       <c r="Q25" t="str">
-        <v>2027-04-28</v>
+        <v>2027-08-28</v>
       </c>
       <c r="R25" t="str">
         <v>Exécuté</v>
@@ -2598,10 +2598,10 @@
         <v>COGS</v>
       </c>
       <c r="P26" t="str">
-        <v>2026-05-01</v>
+        <v>2026-01-01</v>
       </c>
       <c r="Q26" t="str">
-        <v>2026-10-28</v>
+        <v>2026-03-28</v>
       </c>
       <c r="R26" t="str">
         <v>Réalisé</v>
@@ -2684,10 +2684,10 @@
         <v>COGS</v>
       </c>
       <c r="P27" t="str">
-        <v>2026-06-01</v>
+        <v>2026-12-01</v>
       </c>
       <c r="Q27" t="str">
-        <v>2026-12-28</v>
+        <v>2027-06-28</v>
       </c>
       <c r="R27" t="str">
         <v>Identifié</v>
@@ -2770,10 +2770,10 @@
         <v>GA</v>
       </c>
       <c r="P28" t="str">
-        <v>2026-07-01</v>
+        <v>2027-01-01</v>
       </c>
       <c r="Q28" t="str">
-        <v>2027-02-28</v>
+        <v>2028-08-28</v>
       </c>
       <c r="R28" t="str">
         <v>Validé</v>
@@ -2856,10 +2856,10 @@
         <v>REV</v>
       </c>
       <c r="P29" t="str">
-        <v>2026-08-01</v>
+        <v>2026-09-01</v>
       </c>
       <c r="Q29" t="str">
-        <v>2027-04-28</v>
+        <v>2027-05-28</v>
       </c>
       <c r="R29" t="str">
         <v>Planifié</v>
@@ -2942,10 +2942,10 @@
         <v>SGA</v>
       </c>
       <c r="P30" t="str">
-        <v>2026-09-01</v>
+        <v>2026-05-01</v>
       </c>
       <c r="Q30" t="str">
-        <v>2027-06-28</v>
+        <v>2027-04-28</v>
       </c>
       <c r="R30" t="str">
         <v>Exécuté</v>
@@ -3028,10 +3028,10 @@
         <v>COGS</v>
       </c>
       <c r="P31" t="str">
-        <v>2026-10-01</v>
+        <v>2026-05-01</v>
       </c>
       <c r="Q31" t="str">
-        <v>2027-08-28</v>
+        <v>2026-08-28</v>
       </c>
       <c r="R31" t="str">
         <v>Réalisé</v>
@@ -3109,10 +3109,10 @@
         <v>Isabelle Roy</v>
       </c>
       <c r="D2" t="str">
-        <v>2026-01-01</v>
+        <v>2026-11-01</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-03-22</v>
+        <v>2027-01-20</v>
       </c>
       <c r="F2" t="str">
         <v>À faire</v>
@@ -3129,10 +3129,10 @@
         <v>Isabelle Roy</v>
       </c>
       <c r="D3" t="str">
-        <v>2026-03-31</v>
+        <v>2027-01-29</v>
       </c>
       <c r="E3" t="str">
-        <v>2026-06-28</v>
+        <v>2027-04-28</v>
       </c>
       <c r="F3" t="str">
         <v>À faire</v>
@@ -3149,10 +3149,10 @@
         <v>Thomas Petit</v>
       </c>
       <c r="D4" t="str">
-        <v>2026-02-01</v>
+        <v>2026-12-01</v>
       </c>
       <c r="E4" t="str">
-        <v>2026-05-05</v>
+        <v>2027-03-05</v>
       </c>
       <c r="F4" t="str">
         <v>À faire</v>
@@ -3169,10 +3169,10 @@
         <v>Thomas Petit</v>
       </c>
       <c r="D5" t="str">
-        <v>2026-05-16</v>
+        <v>2027-03-15</v>
       </c>
       <c r="E5" t="str">
-        <v>2026-08-28</v>
+        <v>2027-06-28</v>
       </c>
       <c r="F5" t="str">
         <v>À faire</v>
@@ -3189,10 +3189,10 @@
         <v>Claire Fontaine</v>
       </c>
       <c r="D6" t="str">
-        <v>2026-03-01</v>
+        <v>2026-11-01</v>
       </c>
       <c r="E6" t="str">
-        <v>2026-06-17</v>
+        <v>2027-02-16</v>
       </c>
       <c r="F6" t="str">
         <v>En cours</v>
@@ -3209,10 +3209,10 @@
         <v>Claire Fontaine</v>
       </c>
       <c r="D7" t="str">
-        <v>2026-06-29</v>
+        <v>2027-02-28</v>
       </c>
       <c r="E7" t="str">
-        <v>2026-10-28</v>
+        <v>2027-06-28</v>
       </c>
       <c r="F7" t="str">
         <v>À faire</v>
@@ -3232,7 +3232,7 @@
         <v>2026-04-01</v>
       </c>
       <c r="E8" t="str">
-        <v>2026-07-31</v>
+        <v>2026-08-28</v>
       </c>
       <c r="F8" t="str">
         <v>Terminé</v>
@@ -3249,10 +3249,10 @@
         <v>Nadia Klein</v>
       </c>
       <c r="D9" t="str">
-        <v>2026-08-14</v>
+        <v>2026-09-14</v>
       </c>
       <c r="E9" t="str">
-        <v>2026-12-28</v>
+        <v>2027-02-28</v>
       </c>
       <c r="F9" t="str">
         <v>En cours</v>
@@ -3272,7 +3272,7 @@
         <v>2026-05-01</v>
       </c>
       <c r="E10" t="str">
-        <v>2026-09-14</v>
+        <v>2026-06-09</v>
       </c>
       <c r="F10" t="str">
         <v>Terminé</v>
@@ -3289,10 +3289,10 @@
         <v>Elena Ruiz</v>
       </c>
       <c r="D11" t="str">
-        <v>2026-09-29</v>
+        <v>2026-06-14</v>
       </c>
       <c r="E11" t="str">
-        <v>2027-02-28</v>
+        <v>2026-07-28</v>
       </c>
       <c r="F11" t="str">
         <v>Terminé</v>
@@ -3309,10 +3309,10 @@
         <v>Ryan Cole</v>
       </c>
       <c r="D12" t="str">
-        <v>2026-06-01</v>
+        <v>2027-01-01</v>
       </c>
       <c r="E12" t="str">
-        <v>2026-10-27</v>
+        <v>2027-11-10</v>
       </c>
       <c r="F12" t="str">
         <v>À faire</v>
@@ -3329,10 +3329,10 @@
         <v>Ryan Cole</v>
       </c>
       <c r="D13" t="str">
-        <v>2026-11-13</v>
+        <v>2027-12-15</v>
       </c>
       <c r="E13" t="str">
-        <v>2027-04-28</v>
+        <v>2028-11-28</v>
       </c>
       <c r="F13" t="str">
         <v>À faire</v>
@@ -3349,10 +3349,10 @@
         <v>Marc Dubois</v>
       </c>
       <c r="D14" t="str">
-        <v>2026-07-01</v>
+        <v>2026-11-01</v>
       </c>
       <c r="E14" t="str">
-        <v>2026-12-10</v>
+        <v>2027-01-20</v>
       </c>
       <c r="F14" t="str">
         <v>À faire</v>
@@ -3369,10 +3369,10 @@
         <v>Marc Dubois</v>
       </c>
       <c r="D15" t="str">
-        <v>2026-12-29</v>
+        <v>2027-01-29</v>
       </c>
       <c r="E15" t="str">
-        <v>2027-06-28</v>
+        <v>2027-04-28</v>
       </c>
       <c r="F15" t="str">
         <v>À faire</v>
@@ -3389,10 +3389,10 @@
         <v>Léa Moreau</v>
       </c>
       <c r="D16" t="str">
-        <v>2026-08-01</v>
+        <v>2026-10-01</v>
       </c>
       <c r="E16" t="str">
-        <v>2027-01-24</v>
+        <v>2027-01-03</v>
       </c>
       <c r="F16" t="str">
         <v>En cours</v>
@@ -3409,10 +3409,10 @@
         <v>Léa Moreau</v>
       </c>
       <c r="D17" t="str">
-        <v>2027-02-13</v>
+        <v>2027-01-13</v>
       </c>
       <c r="E17" t="str">
-        <v>2027-08-28</v>
+        <v>2027-04-28</v>
       </c>
       <c r="F17" t="str">
         <v>À faire</v>
@@ -3429,10 +3429,10 @@
         <v>Julien Blanc</v>
       </c>
       <c r="D18" t="str">
-        <v>2026-09-01</v>
+        <v>2026-01-01</v>
       </c>
       <c r="E18" t="str">
-        <v>2026-11-21</v>
+        <v>2026-05-16</v>
       </c>
       <c r="F18" t="str">
         <v>Terminé</v>
@@ -3449,10 +3449,10 @@
         <v>Julien Blanc</v>
       </c>
       <c r="D19" t="str">
-        <v>2026-11-30</v>
+        <v>2026-05-31</v>
       </c>
       <c r="E19" t="str">
-        <v>2027-02-28</v>
+        <v>2026-10-28</v>
       </c>
       <c r="F19" t="str">
         <v>En cours</v>
@@ -3469,10 +3469,10 @@
         <v>Sofia Alvarez</v>
       </c>
       <c r="D20" t="str">
-        <v>2026-10-01</v>
+        <v>2026-03-01</v>
       </c>
       <c r="E20" t="str">
-        <v>2027-01-03</v>
+        <v>2026-04-23</v>
       </c>
       <c r="F20" t="str">
         <v>Terminé</v>
@@ -3489,10 +3489,10 @@
         <v>Sofia Alvarez</v>
       </c>
       <c r="D21" t="str">
-        <v>2027-01-13</v>
+        <v>2026-04-29</v>
       </c>
       <c r="E21" t="str">
-        <v>2027-04-28</v>
+        <v>2026-06-28</v>
       </c>
       <c r="F21" t="str">
         <v>Terminé</v>
@@ -3509,10 +3509,10 @@
         <v>Henrik Dahl</v>
       </c>
       <c r="D22" t="str">
-        <v>2026-01-01</v>
+        <v>2026-12-01</v>
       </c>
       <c r="E22" t="str">
-        <v>2026-04-18</v>
+        <v>2027-04-15</v>
       </c>
       <c r="F22" t="str">
         <v>À faire</v>
@@ -3529,10 +3529,10 @@
         <v>Henrik Dahl</v>
       </c>
       <c r="D23" t="str">
-        <v>2026-04-30</v>
+        <v>2027-04-30</v>
       </c>
       <c r="E23" t="str">
-        <v>2026-08-28</v>
+        <v>2027-09-28</v>
       </c>
       <c r="F23" t="str">
         <v>À faire</v>
@@ -3549,10 +3549,10 @@
         <v>Camille Vasseur</v>
       </c>
       <c r="D24" t="str">
-        <v>2026-02-01</v>
+        <v>2027-01-01</v>
       </c>
       <c r="E24" t="str">
-        <v>2026-06-02</v>
+        <v>2027-11-10</v>
       </c>
       <c r="F24" t="str">
         <v>À faire</v>
@@ -3569,10 +3569,10 @@
         <v>Camille Vasseur</v>
       </c>
       <c r="D25" t="str">
-        <v>2026-06-15</v>
+        <v>2027-12-15</v>
       </c>
       <c r="E25" t="str">
-        <v>2026-10-28</v>
+        <v>2028-11-28</v>
       </c>
       <c r="F25" t="str">
         <v>À faire</v>
@@ -3589,10 +3589,10 @@
         <v>Isabelle Roy</v>
       </c>
       <c r="D26" t="str">
-        <v>2026-03-01</v>
+        <v>2026-09-01</v>
       </c>
       <c r="E26" t="str">
-        <v>2026-07-14</v>
+        <v>2026-11-21</v>
       </c>
       <c r="F26" t="str">
         <v>En cours</v>
@@ -3609,10 +3609,10 @@
         <v>Isabelle Roy</v>
       </c>
       <c r="D27" t="str">
-        <v>2026-07-30</v>
+        <v>2026-11-30</v>
       </c>
       <c r="E27" t="str">
-        <v>2026-12-28</v>
+        <v>2027-02-28</v>
       </c>
       <c r="F27" t="str">
         <v>À faire</v>
@@ -3629,10 +3629,10 @@
         <v>Thomas Petit</v>
       </c>
       <c r="D28" t="str">
-        <v>2026-04-01</v>
+        <v>2026-06-01</v>
       </c>
       <c r="E28" t="str">
-        <v>2026-08-28</v>
+        <v>2026-10-01</v>
       </c>
       <c r="F28" t="str">
         <v>Terminé</v>
@@ -3649,7 +3649,7 @@
         <v>Thomas Petit</v>
       </c>
       <c r="D29" t="str">
-        <v>2026-09-14</v>
+        <v>2026-10-15</v>
       </c>
       <c r="E29" t="str">
         <v>2027-02-28</v>
@@ -3669,10 +3669,10 @@
         <v>Claire Fontaine</v>
       </c>
       <c r="D30" t="str">
-        <v>2026-05-01</v>
+        <v>2026-01-01</v>
       </c>
       <c r="E30" t="str">
-        <v>2026-10-10</v>
+        <v>2026-03-08</v>
       </c>
       <c r="F30" t="str">
         <v>Terminé</v>
@@ -3689,10 +3689,10 @@
         <v>Claire Fontaine</v>
       </c>
       <c r="D31" t="str">
-        <v>2026-10-29</v>
+        <v>2026-03-15</v>
       </c>
       <c r="E31" t="str">
-        <v>2027-04-28</v>
+        <v>2026-05-28</v>
       </c>
       <c r="F31" t="str">
         <v>Terminé</v>
@@ -3709,10 +3709,10 @@
         <v>Nadia Klein</v>
       </c>
       <c r="D32" t="str">
-        <v>2026-06-01</v>
+        <v>2026-11-01</v>
       </c>
       <c r="E32" t="str">
-        <v>2026-11-24</v>
+        <v>2027-03-02</v>
       </c>
       <c r="F32" t="str">
         <v>À faire</v>
@@ -3729,10 +3729,10 @@
         <v>Nadia Klein</v>
       </c>
       <c r="D33" t="str">
-        <v>2026-12-14</v>
+        <v>2027-03-15</v>
       </c>
       <c r="E33" t="str">
-        <v>2027-06-28</v>
+        <v>2027-07-28</v>
       </c>
       <c r="F33" t="str">
         <v>À faire</v>
@@ -3749,10 +3749,10 @@
         <v>Elena Ruiz</v>
       </c>
       <c r="D34" t="str">
-        <v>2026-07-01</v>
+        <v>2026-12-01</v>
       </c>
       <c r="E34" t="str">
-        <v>2026-09-20</v>
+        <v>2027-04-15</v>
       </c>
       <c r="F34" t="str">
         <v>À faire</v>
@@ -3769,10 +3769,10 @@
         <v>Elena Ruiz</v>
       </c>
       <c r="D35" t="str">
-        <v>2026-09-29</v>
+        <v>2027-04-30</v>
       </c>
       <c r="E35" t="str">
-        <v>2026-12-28</v>
+        <v>2027-09-28</v>
       </c>
       <c r="F35" t="str">
         <v>À faire</v>
@@ -3789,10 +3789,10 @@
         <v>Ryan Cole</v>
       </c>
       <c r="D36" t="str">
-        <v>2026-08-01</v>
+        <v>2026-11-01</v>
       </c>
       <c r="E36" t="str">
-        <v>2026-11-03</v>
+        <v>2027-03-29</v>
       </c>
       <c r="F36" t="str">
         <v>En cours</v>
@@ -3809,10 +3809,10 @@
         <v>Ryan Cole</v>
       </c>
       <c r="D37" t="str">
-        <v>2026-11-14</v>
+        <v>2027-04-15</v>
       </c>
       <c r="E37" t="str">
-        <v>2027-02-28</v>
+        <v>2027-09-28</v>
       </c>
       <c r="F37" t="str">
         <v>À faire</v>
@@ -3829,10 +3829,10 @@
         <v>Marc Dubois</v>
       </c>
       <c r="D38" t="str">
-        <v>2026-09-01</v>
+        <v>2026-03-01</v>
       </c>
       <c r="E38" t="str">
-        <v>2026-12-17</v>
+        <v>2026-06-17</v>
       </c>
       <c r="F38" t="str">
         <v>En cours</v>
@@ -3849,10 +3849,10 @@
         <v>Marc Dubois</v>
       </c>
       <c r="D39" t="str">
-        <v>2026-12-29</v>
+        <v>2026-06-29</v>
       </c>
       <c r="E39" t="str">
-        <v>2027-04-28</v>
+        <v>2026-10-28</v>
       </c>
       <c r="F39" t="str">
         <v>À faire</v>
@@ -3869,10 +3869,10 @@
         <v>Léa Moreau</v>
       </c>
       <c r="D40" t="str">
-        <v>2026-10-01</v>
+        <v>2026-01-01</v>
       </c>
       <c r="E40" t="str">
-        <v>2027-01-30</v>
+        <v>2026-03-22</v>
       </c>
       <c r="F40" t="str">
         <v>Terminé</v>
@@ -3889,10 +3889,10 @@
         <v>Léa Moreau</v>
       </c>
       <c r="D41" t="str">
-        <v>2027-02-13</v>
+        <v>2026-03-31</v>
       </c>
       <c r="E41" t="str">
-        <v>2027-06-28</v>
+        <v>2026-06-28</v>
       </c>
       <c r="F41" t="str">
         <v>Terminé</v>
@@ -3909,10 +3909,10 @@
         <v>Julien Blanc</v>
       </c>
       <c r="D42" t="str">
-        <v>2026-01-01</v>
+        <v>2027-01-01</v>
       </c>
       <c r="E42" t="str">
-        <v>2026-05-16</v>
+        <v>2027-09-30</v>
       </c>
       <c r="F42" t="str">
         <v>À faire</v>
@@ -3929,10 +3929,10 @@
         <v>Julien Blanc</v>
       </c>
       <c r="D43" t="str">
-        <v>2026-05-31</v>
+        <v>2027-10-30</v>
       </c>
       <c r="E43" t="str">
-        <v>2026-10-28</v>
+        <v>2028-08-28</v>
       </c>
       <c r="F43" t="str">
         <v>À faire</v>
@@ -3949,10 +3949,10 @@
         <v>Sofia Alvarez</v>
       </c>
       <c r="D44" t="str">
-        <v>2026-02-01</v>
+        <v>2026-11-01</v>
       </c>
       <c r="E44" t="str">
-        <v>2026-06-29</v>
+        <v>2027-03-02</v>
       </c>
       <c r="F44" t="str">
         <v>À faire</v>
@@ -3969,10 +3969,10 @@
         <v>Sofia Alvarez</v>
       </c>
       <c r="D45" t="str">
-        <v>2026-07-16</v>
+        <v>2027-03-15</v>
       </c>
       <c r="E45" t="str">
-        <v>2026-12-28</v>
+        <v>2027-07-28</v>
       </c>
       <c r="F45" t="str">
         <v>À faire</v>
@@ -3989,10 +3989,10 @@
         <v>Henrik Dahl</v>
       </c>
       <c r="D46" t="str">
-        <v>2026-03-01</v>
+        <v>2026-10-01</v>
       </c>
       <c r="E46" t="str">
-        <v>2026-08-11</v>
+        <v>2027-02-13</v>
       </c>
       <c r="F46" t="str">
         <v>En cours</v>
@@ -4009,10 +4009,10 @@
         <v>Henrik Dahl</v>
       </c>
       <c r="D47" t="str">
-        <v>2026-08-30</v>
+        <v>2027-02-28</v>
       </c>
       <c r="E47" t="str">
-        <v>2027-02-28</v>
+        <v>2027-07-28</v>
       </c>
       <c r="F47" t="str">
         <v>À faire</v>
@@ -4029,10 +4029,10 @@
         <v>Camille Vasseur</v>
       </c>
       <c r="D48" t="str">
-        <v>2026-04-01</v>
+        <v>2026-08-01</v>
       </c>
       <c r="E48" t="str">
-        <v>2026-09-24</v>
+        <v>2027-01-24</v>
       </c>
       <c r="F48" t="str">
         <v>Terminé</v>
@@ -4049,10 +4049,10 @@
         <v>Camille Vasseur</v>
       </c>
       <c r="D49" t="str">
-        <v>2026-10-14</v>
+        <v>2027-02-13</v>
       </c>
       <c r="E49" t="str">
-        <v>2027-04-28</v>
+        <v>2027-08-28</v>
       </c>
       <c r="F49" t="str">
         <v>Terminé</v>
@@ -4069,10 +4069,10 @@
         <v>Isabelle Roy</v>
       </c>
       <c r="D50" t="str">
-        <v>2026-05-01</v>
+        <v>2026-01-01</v>
       </c>
       <c r="E50" t="str">
-        <v>2026-07-21</v>
+        <v>2026-02-08</v>
       </c>
       <c r="F50" t="str">
         <v>Terminé</v>
@@ -4089,10 +4089,10 @@
         <v>Isabelle Roy</v>
       </c>
       <c r="D51" t="str">
-        <v>2026-07-30</v>
+        <v>2026-02-13</v>
       </c>
       <c r="E51" t="str">
-        <v>2026-10-28</v>
+        <v>2026-03-28</v>
       </c>
       <c r="F51" t="str">
         <v>Terminé</v>
@@ -4109,10 +4109,10 @@
         <v>Thomas Petit</v>
       </c>
       <c r="D52" t="str">
-        <v>2026-06-01</v>
+        <v>2026-12-01</v>
       </c>
       <c r="E52" t="str">
-        <v>2026-09-03</v>
+        <v>2027-03-05</v>
       </c>
       <c r="F52" t="str">
         <v>À faire</v>
@@ -4129,10 +4129,10 @@
         <v>Thomas Petit</v>
       </c>
       <c r="D53" t="str">
-        <v>2026-09-14</v>
+        <v>2027-03-15</v>
       </c>
       <c r="E53" t="str">
-        <v>2026-12-28</v>
+        <v>2027-06-28</v>
       </c>
       <c r="F53" t="str">
         <v>À faire</v>
@@ -4149,10 +4149,10 @@
         <v>Claire Fontaine</v>
       </c>
       <c r="D54" t="str">
-        <v>2026-07-01</v>
+        <v>2027-01-01</v>
       </c>
       <c r="E54" t="str">
-        <v>2026-10-17</v>
+        <v>2027-09-30</v>
       </c>
       <c r="F54" t="str">
         <v>À faire</v>
@@ -4169,10 +4169,10 @@
         <v>Claire Fontaine</v>
       </c>
       <c r="D55" t="str">
-        <v>2026-10-30</v>
+        <v>2027-10-30</v>
       </c>
       <c r="E55" t="str">
-        <v>2027-02-28</v>
+        <v>2028-08-28</v>
       </c>
       <c r="F55" t="str">
         <v>À faire</v>
@@ -4189,10 +4189,10 @@
         <v>Nadia Klein</v>
       </c>
       <c r="D56" t="str">
-        <v>2026-08-01</v>
+        <v>2026-09-01</v>
       </c>
       <c r="E56" t="str">
-        <v>2026-11-30</v>
+        <v>2026-12-31</v>
       </c>
       <c r="F56" t="str">
         <v>En cours</v>
@@ -4209,10 +4209,10 @@
         <v>Nadia Klein</v>
       </c>
       <c r="D57" t="str">
-        <v>2026-12-14</v>
+        <v>2027-01-13</v>
       </c>
       <c r="E57" t="str">
-        <v>2027-04-28</v>
+        <v>2027-05-28</v>
       </c>
       <c r="F57" t="str">
         <v>À faire</v>
@@ -4229,10 +4229,10 @@
         <v>Elena Ruiz</v>
       </c>
       <c r="D58" t="str">
-        <v>2026-09-01</v>
+        <v>2026-05-01</v>
       </c>
       <c r="E58" t="str">
-        <v>2027-01-14</v>
+        <v>2026-10-10</v>
       </c>
       <c r="F58" t="str">
         <v>Terminé</v>
@@ -4249,10 +4249,10 @@
         <v>Elena Ruiz</v>
       </c>
       <c r="D59" t="str">
-        <v>2027-01-29</v>
+        <v>2026-10-29</v>
       </c>
       <c r="E59" t="str">
-        <v>2027-06-28</v>
+        <v>2027-04-28</v>
       </c>
       <c r="F59" t="str">
         <v>En cours</v>
@@ -4269,10 +4269,10 @@
         <v>Ryan Cole</v>
       </c>
       <c r="D60" t="str">
-        <v>2026-10-01</v>
+        <v>2026-05-01</v>
       </c>
       <c r="E60" t="str">
-        <v>2027-02-26</v>
+        <v>2026-06-23</v>
       </c>
       <c r="F60" t="str">
         <v>Terminé</v>
@@ -4289,10 +4289,10 @@
         <v>Ryan Cole</v>
       </c>
       <c r="D61" t="str">
-        <v>2027-03-15</v>
+        <v>2026-06-29</v>
       </c>
       <c r="E61" t="str">
-        <v>2027-08-28</v>
+        <v>2026-08-28</v>
       </c>
       <c r="F61" t="str">
         <v>Terminé</v>
@@ -4376,7 +4376,7 @@
         <v/>
       </c>
       <c r="H2" t="str">
-        <v>2026-03-22</v>
+        <v>2027-01-20</v>
       </c>
       <c r="I2" t="str">
         <v/>
@@ -4511,7 +4511,7 @@
         <v/>
       </c>
       <c r="I5" t="str">
-        <v>2026-06-28</v>
+        <v>2027-04-28</v>
       </c>
       <c r="J5" t="str">
         <v/>
@@ -4552,7 +4552,7 @@
         <v/>
       </c>
       <c r="H6" t="str">
-        <v>2026-05-05</v>
+        <v>2027-03-05</v>
       </c>
       <c r="I6" t="str">
         <v/>
@@ -4687,7 +4687,7 @@
         <v/>
       </c>
       <c r="I9" t="str">
-        <v>2026-08-28</v>
+        <v>2027-06-28</v>
       </c>
       <c r="J9" t="str">
         <v/>
@@ -4728,7 +4728,7 @@
         <v/>
       </c>
       <c r="H10" t="str">
-        <v>2026-06-17</v>
+        <v>2027-02-16</v>
       </c>
       <c r="I10" t="str">
         <v/>
@@ -4863,7 +4863,7 @@
         <v/>
       </c>
       <c r="I13" t="str">
-        <v>2026-10-28</v>
+        <v>2027-06-28</v>
       </c>
       <c r="J13" t="str">
         <v/>
@@ -4904,7 +4904,7 @@
         <v/>
       </c>
       <c r="H14" t="str">
-        <v>2026-07-31</v>
+        <v>2026-08-28</v>
       </c>
       <c r="I14" t="str">
         <v/>
@@ -5039,7 +5039,7 @@
         <v/>
       </c>
       <c r="I17" t="str">
-        <v>2026-12-28</v>
+        <v>2027-02-28</v>
       </c>
       <c r="J17" t="str">
         <v/>
@@ -5080,7 +5080,7 @@
         <v/>
       </c>
       <c r="H18" t="str">
-        <v>2026-09-14</v>
+        <v>2026-06-09</v>
       </c>
       <c r="I18" t="str">
         <v/>
@@ -5215,7 +5215,7 @@
         <v/>
       </c>
       <c r="I21" t="str">
-        <v>2027-02-28</v>
+        <v>2026-07-28</v>
       </c>
       <c r="J21" t="str">
         <v/>
@@ -5256,7 +5256,7 @@
         <v/>
       </c>
       <c r="H22" t="str">
-        <v>2026-10-27</v>
+        <v>2027-11-10</v>
       </c>
       <c r="I22" t="str">
         <v/>
@@ -5391,7 +5391,7 @@
         <v/>
       </c>
       <c r="I25" t="str">
-        <v>2027-04-28</v>
+        <v>2028-11-28</v>
       </c>
       <c r="J25" t="str">
         <v/>
@@ -5432,7 +5432,7 @@
         <v/>
       </c>
       <c r="H26" t="str">
-        <v>2026-12-10</v>
+        <v>2027-01-20</v>
       </c>
       <c r="I26" t="str">
         <v/>
@@ -5567,7 +5567,7 @@
         <v/>
       </c>
       <c r="I29" t="str">
-        <v>2027-06-28</v>
+        <v>2027-04-28</v>
       </c>
       <c r="J29" t="str">
         <v/>
@@ -5608,7 +5608,7 @@
         <v/>
       </c>
       <c r="H30" t="str">
-        <v>2027-01-24</v>
+        <v>2027-01-03</v>
       </c>
       <c r="I30" t="str">
         <v/>
@@ -5743,7 +5743,7 @@
         <v/>
       </c>
       <c r="I33" t="str">
-        <v>2027-08-28</v>
+        <v>2027-04-28</v>
       </c>
       <c r="J33" t="str">
         <v/>
@@ -5784,7 +5784,7 @@
         <v/>
       </c>
       <c r="H34" t="str">
-        <v>2026-11-21</v>
+        <v>2026-05-16</v>
       </c>
       <c r="I34" t="str">
         <v/>
@@ -5919,7 +5919,7 @@
         <v/>
       </c>
       <c r="I37" t="str">
-        <v>2027-02-28</v>
+        <v>2026-10-28</v>
       </c>
       <c r="J37" t="str">
         <v/>
@@ -5960,7 +5960,7 @@
         <v/>
       </c>
       <c r="H38" t="str">
-        <v>2027-01-03</v>
+        <v>2026-04-23</v>
       </c>
       <c r="I38" t="str">
         <v/>
@@ -6095,7 +6095,7 @@
         <v/>
       </c>
       <c r="I41" t="str">
-        <v>2027-04-28</v>
+        <v>2026-06-28</v>
       </c>
       <c r="J41" t="str">
         <v/>
@@ -6136,7 +6136,7 @@
         <v/>
       </c>
       <c r="H42" t="str">
-        <v>2026-04-18</v>
+        <v>2027-04-15</v>
       </c>
       <c r="I42" t="str">
         <v/>
@@ -6271,7 +6271,7 @@
         <v/>
       </c>
       <c r="I45" t="str">
-        <v>2026-08-28</v>
+        <v>2027-09-28</v>
       </c>
       <c r="J45" t="str">
         <v/>
@@ -6312,7 +6312,7 @@
         <v/>
       </c>
       <c r="H46" t="str">
-        <v>2026-06-02</v>
+        <v>2027-11-10</v>
       </c>
       <c r="I46" t="str">
         <v/>
@@ -6447,7 +6447,7 @@
         <v/>
       </c>
       <c r="I49" t="str">
-        <v>2026-10-28</v>
+        <v>2028-11-28</v>
       </c>
       <c r="J49" t="str">
         <v/>
@@ -6488,7 +6488,7 @@
         <v/>
       </c>
       <c r="H50" t="str">
-        <v>2026-07-14</v>
+        <v>2026-11-21</v>
       </c>
       <c r="I50" t="str">
         <v/>
@@ -6623,7 +6623,7 @@
         <v/>
       </c>
       <c r="I53" t="str">
-        <v>2026-12-28</v>
+        <v>2027-02-28</v>
       </c>
       <c r="J53" t="str">
         <v/>
@@ -6664,7 +6664,7 @@
         <v/>
       </c>
       <c r="H54" t="str">
-        <v>2026-08-28</v>
+        <v>2026-10-01</v>
       </c>
       <c r="I54" t="str">
         <v/>
@@ -6840,7 +6840,7 @@
         <v/>
       </c>
       <c r="H58" t="str">
-        <v>2026-10-10</v>
+        <v>2026-03-08</v>
       </c>
       <c r="I58" t="str">
         <v/>
@@ -6975,7 +6975,7 @@
         <v/>
       </c>
       <c r="I61" t="str">
-        <v>2027-04-28</v>
+        <v>2026-05-28</v>
       </c>
       <c r="J61" t="str">
         <v/>
@@ -7016,7 +7016,7 @@
         <v/>
       </c>
       <c r="H62" t="str">
-        <v>2026-11-24</v>
+        <v>2027-03-02</v>
       </c>
       <c r="I62" t="str">
         <v/>
@@ -7151,7 +7151,7 @@
         <v/>
       </c>
       <c r="I65" t="str">
-        <v>2027-06-28</v>
+        <v>2027-07-28</v>
       </c>
       <c r="J65" t="str">
         <v/>
@@ -7192,7 +7192,7 @@
         <v/>
       </c>
       <c r="H66" t="str">
-        <v>2026-09-20</v>
+        <v>2027-04-15</v>
       </c>
       <c r="I66" t="str">
         <v/>
@@ -7327,7 +7327,7 @@
         <v/>
       </c>
       <c r="I69" t="str">
-        <v>2026-12-28</v>
+        <v>2027-09-28</v>
       </c>
       <c r="J69" t="str">
         <v/>
@@ -7368,7 +7368,7 @@
         <v/>
       </c>
       <c r="H70" t="str">
-        <v>2026-11-03</v>
+        <v>2027-03-29</v>
       </c>
       <c r="I70" t="str">
         <v/>
@@ -7503,7 +7503,7 @@
         <v/>
       </c>
       <c r="I73" t="str">
-        <v>2027-02-28</v>
+        <v>2027-09-28</v>
       </c>
       <c r="J73" t="str">
         <v/>
@@ -7544,7 +7544,7 @@
         <v/>
       </c>
       <c r="H74" t="str">
-        <v>2026-12-17</v>
+        <v>2026-06-17</v>
       </c>
       <c r="I74" t="str">
         <v/>
@@ -7679,7 +7679,7 @@
         <v/>
       </c>
       <c r="I77" t="str">
-        <v>2027-04-28</v>
+        <v>2026-10-28</v>
       </c>
       <c r="J77" t="str">
         <v/>
@@ -7720,7 +7720,7 @@
         <v/>
       </c>
       <c r="H78" t="str">
-        <v>2027-01-30</v>
+        <v>2026-03-22</v>
       </c>
       <c r="I78" t="str">
         <v/>
@@ -7855,7 +7855,7 @@
         <v/>
       </c>
       <c r="I81" t="str">
-        <v>2027-06-28</v>
+        <v>2026-06-28</v>
       </c>
       <c r="J81" t="str">
         <v/>
@@ -7896,7 +7896,7 @@
         <v/>
       </c>
       <c r="H82" t="str">
-        <v>2026-05-16</v>
+        <v>2027-09-30</v>
       </c>
       <c r="I82" t="str">
         <v/>
@@ -8031,7 +8031,7 @@
         <v/>
       </c>
       <c r="I85" t="str">
-        <v>2026-10-28</v>
+        <v>2028-08-28</v>
       </c>
       <c r="J85" t="str">
         <v/>
@@ -8072,7 +8072,7 @@
         <v/>
       </c>
       <c r="H86" t="str">
-        <v>2026-06-29</v>
+        <v>2027-03-02</v>
       </c>
       <c r="I86" t="str">
         <v/>
@@ -8207,7 +8207,7 @@
         <v/>
       </c>
       <c r="I89" t="str">
-        <v>2026-12-28</v>
+        <v>2027-07-28</v>
       </c>
       <c r="J89" t="str">
         <v/>
@@ -8248,7 +8248,7 @@
         <v/>
       </c>
       <c r="H90" t="str">
-        <v>2026-08-11</v>
+        <v>2027-02-13</v>
       </c>
       <c r="I90" t="str">
         <v/>
@@ -8383,7 +8383,7 @@
         <v/>
       </c>
       <c r="I93" t="str">
-        <v>2027-02-28</v>
+        <v>2027-07-28</v>
       </c>
       <c r="J93" t="str">
         <v/>
@@ -8424,7 +8424,7 @@
         <v/>
       </c>
       <c r="H94" t="str">
-        <v>2026-09-24</v>
+        <v>2027-01-24</v>
       </c>
       <c r="I94" t="str">
         <v/>
@@ -8559,7 +8559,7 @@
         <v/>
       </c>
       <c r="I97" t="str">
-        <v>2027-04-28</v>
+        <v>2027-08-28</v>
       </c>
       <c r="J97" t="str">
         <v/>
@@ -8600,7 +8600,7 @@
         <v/>
       </c>
       <c r="H98" t="str">
-        <v>2026-07-21</v>
+        <v>2026-02-08</v>
       </c>
       <c r="I98" t="str">
         <v/>
@@ -8735,7 +8735,7 @@
         <v/>
       </c>
       <c r="I101" t="str">
-        <v>2026-10-28</v>
+        <v>2026-03-28</v>
       </c>
       <c r="J101" t="str">
         <v/>
@@ -8776,7 +8776,7 @@
         <v/>
       </c>
       <c r="H102" t="str">
-        <v>2026-09-03</v>
+        <v>2027-03-05</v>
       </c>
       <c r="I102" t="str">
         <v/>
@@ -8911,7 +8911,7 @@
         <v/>
       </c>
       <c r="I105" t="str">
-        <v>2026-12-28</v>
+        <v>2027-06-28</v>
       </c>
       <c r="J105" t="str">
         <v/>
@@ -8952,7 +8952,7 @@
         <v/>
       </c>
       <c r="H106" t="str">
-        <v>2026-10-17</v>
+        <v>2027-09-30</v>
       </c>
       <c r="I106" t="str">
         <v/>
@@ -9087,7 +9087,7 @@
         <v/>
       </c>
       <c r="I109" t="str">
-        <v>2027-02-28</v>
+        <v>2028-08-28</v>
       </c>
       <c r="J109" t="str">
         <v/>
@@ -9128,7 +9128,7 @@
         <v/>
       </c>
       <c r="H110" t="str">
-        <v>2026-11-30</v>
+        <v>2026-12-31</v>
       </c>
       <c r="I110" t="str">
         <v/>
@@ -9263,7 +9263,7 @@
         <v/>
       </c>
       <c r="I113" t="str">
-        <v>2027-04-28</v>
+        <v>2027-05-28</v>
       </c>
       <c r="J113" t="str">
         <v/>
@@ -9304,7 +9304,7 @@
         <v/>
       </c>
       <c r="H114" t="str">
-        <v>2027-01-14</v>
+        <v>2026-10-10</v>
       </c>
       <c r="I114" t="str">
         <v/>
@@ -9439,7 +9439,7 @@
         <v/>
       </c>
       <c r="I117" t="str">
-        <v>2027-06-28</v>
+        <v>2027-04-28</v>
       </c>
       <c r="J117" t="str">
         <v/>
@@ -9480,7 +9480,7 @@
         <v/>
       </c>
       <c r="H118" t="str">
-        <v>2027-02-26</v>
+        <v>2026-06-23</v>
       </c>
       <c r="I118" t="str">
         <v/>
@@ -9615,7 +9615,7 @@
         <v/>
       </c>
       <c r="I121" t="str">
-        <v>2027-08-28</v>
+        <v>2026-08-28</v>
       </c>
       <c r="J121" t="str">
         <v/>

</xml_diff>